<commit_message>
Update analysis files and add regression plots for sunshine and evaporation data
- Modified the following Excel files:
  - `evaporation_frequency_distribution.xlsx`
  - `evaporation_mean_calculation.xlsx`
  - `regression_table.xlsx`
  - `sunshine_frequency_distribution.xlsx`
  - `sunshine_mean_calculation.xlsx`
  - Added new `correlation_table.xlsx`

- Added regression plot images:
  - `regression_plot_sunshine_evaporation.png`
  - `scatter_plot_sunshine_evaporation.png`
</commit_message>
<xml_diff>
--- a/regression_table.xlsx
+++ b/regression_table.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F101"/>
+  <dimension ref="A1:I101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,6 +459,21 @@
           <t>XY</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Y_predicted</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Residual (Y - Y_pred)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Residual^2</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -479,6 +494,15 @@
       <c r="F2" t="n">
         <v>0</v>
       </c>
+      <c r="G2" t="n">
+        <v>4.249371858230057</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1.950628141769943</v>
+      </c>
+      <c r="I2" t="n">
+        <v>3.804950147464862</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -499,6 +523,15 @@
       <c r="F3" t="n">
         <v>9.18</v>
       </c>
+      <c r="G3" t="n">
+        <v>4.483614185782558</v>
+      </c>
+      <c r="H3" t="n">
+        <v>-1.083614185782559</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1.174219703629197</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -519,6 +552,15 @@
       <c r="F4" t="n">
         <v>0.24</v>
       </c>
+      <c r="G4" t="n">
+        <v>4.25804749999126</v>
+      </c>
+      <c r="H4" t="n">
+        <v>-1.85804749999126</v>
+      </c>
+      <c r="I4" t="n">
+        <v>3.452340512223773</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -539,6 +581,15 @@
       <c r="F5" t="n">
         <v>0</v>
       </c>
+      <c r="G5" t="n">
+        <v>4.249371858230057</v>
+      </c>
+      <c r="H5" t="n">
+        <v>-2.049371858230057</v>
+      </c>
+      <c r="I5" t="n">
+        <v>4.199925013305315</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -559,6 +610,15 @@
       <c r="F6" t="n">
         <v>0</v>
       </c>
+      <c r="G6" t="n">
+        <v>4.249371858230057</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.550628141769943</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.3031913505090205</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -579,6 +639,15 @@
       <c r="F7" t="n">
         <v>22.36</v>
       </c>
+      <c r="G7" t="n">
+        <v>4.995477049693581</v>
+      </c>
+      <c r="H7" t="n">
+        <v>-2.395477049693581</v>
+      </c>
+      <c r="I7" t="n">
+        <v>5.738310295608662</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -599,6 +668,15 @@
       <c r="F8" t="n">
         <v>27.04</v>
       </c>
+      <c r="G8" t="n">
+        <v>4.700505229812653</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.4994947701873471</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.2494950254445107</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -619,6 +697,15 @@
       <c r="F9" t="n">
         <v>12.18</v>
       </c>
+      <c r="G9" t="n">
+        <v>4.431560335215336</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1.368439664784664</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1.872627116155964</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -639,6 +726,15 @@
       <c r="F10" t="n">
         <v>14.4</v>
       </c>
+      <c r="G10" t="n">
+        <v>4.50964111106617</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.29035888893383</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.08430828438288822</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -659,6 +755,15 @@
       <c r="F11" t="n">
         <v>44.44</v>
       </c>
+      <c r="G11" t="n">
+        <v>5.125611676111637</v>
+      </c>
+      <c r="H11" t="n">
+        <v>-0.7256116761116367</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.5265123045095388</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -679,6 +784,15 @@
       <c r="F12" t="n">
         <v>51.2</v>
       </c>
+      <c r="G12" t="n">
+        <v>4.943423199126358</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1.456576800873642</v>
+      </c>
+      <c r="I12" t="n">
+        <v>2.121615976843294</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -699,6 +813,15 @@
       <c r="F13" t="n">
         <v>45.56</v>
       </c>
+      <c r="G13" t="n">
+        <v>4.830639856230709</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1.969360143769291</v>
+      </c>
+      <c r="I13" t="n">
+        <v>3.878379375867001</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -719,6 +842,15 @@
       <c r="F14" t="n">
         <v>23.1</v>
       </c>
+      <c r="G14" t="n">
+        <v>4.535668036349781</v>
+      </c>
+      <c r="H14" t="n">
+        <v>2.464331963650219</v>
+      </c>
+      <c r="I14" t="n">
+        <v>6.072932027068143</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -739,6 +871,15 @@
       <c r="F15" t="n">
         <v>27.84</v>
       </c>
+      <c r="G15" t="n">
+        <v>5.004152691454784</v>
+      </c>
+      <c r="H15" t="n">
+        <v>-1.804152691454784</v>
+      </c>
+      <c r="I15" t="n">
+        <v>3.254966934083542</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -759,6 +900,15 @@
       <c r="F16" t="n">
         <v>52.7</v>
       </c>
+      <c r="G16" t="n">
+        <v>4.986801407932377</v>
+      </c>
+      <c r="H16" t="n">
+        <v>1.213198592067623</v>
+      </c>
+      <c r="I16" t="n">
+        <v>1.471850823794862</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -779,6 +929,15 @@
       <c r="F17" t="n">
         <v>54.56000000000001</v>
       </c>
+      <c r="G17" t="n">
+        <v>5.012828333215989</v>
+      </c>
+      <c r="H17" t="n">
+        <v>1.187171666784011</v>
+      </c>
+      <c r="I17" t="n">
+        <v>1.409376566414728</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -799,6 +958,15 @@
       <c r="F18" t="n">
         <v>24.32</v>
       </c>
+      <c r="G18" t="n">
+        <v>4.526992394588578</v>
+      </c>
+      <c r="H18" t="n">
+        <v>3.073007605411422</v>
+      </c>
+      <c r="I18" t="n">
+        <v>9.443375742916441</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -819,6 +987,15 @@
       <c r="F19" t="n">
         <v>18.9</v>
       </c>
+      <c r="G19" t="n">
+        <v>4.639775737484227</v>
+      </c>
+      <c r="H19" t="n">
+        <v>-0.4397757374842266</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.1934026992797954</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -839,6 +1016,15 @@
       <c r="F20" t="n">
         <v>39</v>
       </c>
+      <c r="G20" t="n">
+        <v>4.90004499032034</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.2999550096796604</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.08997300783192515</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -859,6 +1045,15 @@
       <c r="F21" t="n">
         <v>51.06</v>
       </c>
+      <c r="G21" t="n">
+        <v>5.212368093723676</v>
+      </c>
+      <c r="H21" t="n">
+        <v>-0.612368093723676</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0.3749946822107688</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -879,6 +1074,15 @@
       <c r="F22" t="n">
         <v>43.52</v>
       </c>
+      <c r="G22" t="n">
+        <v>4.804612930947098</v>
+      </c>
+      <c r="H22" t="n">
+        <v>1.995387069052902</v>
+      </c>
+      <c r="I22" t="n">
+        <v>3.981569555343531</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -899,6 +1103,15 @@
       <c r="F23" t="n">
         <v>41.36000000000001</v>
       </c>
+      <c r="G23" t="n">
+        <v>5.064882183783211</v>
+      </c>
+      <c r="H23" t="n">
+        <v>-0.6648821837832104</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0.4420683183123308</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -919,6 +1132,15 @@
       <c r="F24" t="n">
         <v>80.52</v>
       </c>
+      <c r="G24" t="n">
+        <v>5.307800153096917</v>
+      </c>
+      <c r="H24" t="n">
+        <v>1.292199846903083</v>
+      </c>
+      <c r="I24" t="n">
+        <v>1.669780444336351</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -939,6 +1161,15 @@
       <c r="F25" t="n">
         <v>103.2</v>
       </c>
+      <c r="G25" t="n">
+        <v>5.290448869574509</v>
+      </c>
+      <c r="H25" t="n">
+        <v>3.309551130425491</v>
+      </c>
+      <c r="I25" t="n">
+        <v>10.95312868490064</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -959,6 +1190,15 @@
       <c r="F26" t="n">
         <v>12.9</v>
       </c>
+      <c r="G26" t="n">
+        <v>4.379506484648114</v>
+      </c>
+      <c r="H26" t="n">
+        <v>4.220493515351886</v>
+      </c>
+      <c r="I26" t="n">
+        <v>17.81256551312732</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -979,6 +1219,15 @@
       <c r="F27" t="n">
         <v>30.24</v>
       </c>
+      <c r="G27" t="n">
+        <v>4.978125766171173</v>
+      </c>
+      <c r="H27" t="n">
+        <v>-1.378125766171173</v>
+      </c>
+      <c r="I27" t="n">
+        <v>1.899230627384883</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -999,6 +1248,15 @@
       <c r="F28" t="n">
         <v>27.06</v>
       </c>
+      <c r="G28" t="n">
+        <v>4.535668036349781</v>
+      </c>
+      <c r="H28" t="n">
+        <v>3.664331963650218</v>
+      </c>
+      <c r="I28" t="n">
+        <v>13.42732873982866</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1019,6 +1277,15 @@
       <c r="F29" t="n">
         <v>0</v>
       </c>
+      <c r="G29" t="n">
+        <v>4.249371858230057</v>
+      </c>
+      <c r="H29" t="n">
+        <v>-0.04937185823005663</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0.002437580385088811</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1039,6 +1306,15 @@
       <c r="F30" t="n">
         <v>62.3</v>
       </c>
+      <c r="G30" t="n">
+        <v>5.021503974977192</v>
+      </c>
+      <c r="H30" t="n">
+        <v>1.978496025022808</v>
+      </c>
+      <c r="I30" t="n">
+        <v>3.91444652103105</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1059,6 +1335,15 @@
       <c r="F31" t="n">
         <v>70.06</v>
       </c>
+      <c r="G31" t="n">
+        <v>5.229719377246083</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0.9702806227539176</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0.9414444868917301</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1079,6 +1364,15 @@
       <c r="F32" t="n">
         <v>46.72</v>
       </c>
+      <c r="G32" t="n">
+        <v>4.882693706797932</v>
+      </c>
+      <c r="H32" t="n">
+        <v>1.517306293202068</v>
+      </c>
+      <c r="I32" t="n">
+        <v>2.302218387390601</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1099,6 +1393,15 @@
       <c r="F33" t="n">
         <v>29.12</v>
       </c>
+      <c r="G33" t="n">
+        <v>5.221043735484879</v>
+      </c>
+      <c r="H33" t="n">
+        <v>-2.621043735484879</v>
+      </c>
+      <c r="I33" t="n">
+        <v>6.869870263324528</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1119,6 +1422,15 @@
       <c r="F34" t="n">
         <v>76.84</v>
       </c>
+      <c r="G34" t="n">
+        <v>5.229719377246083</v>
+      </c>
+      <c r="H34" t="n">
+        <v>1.570280622753917</v>
+      </c>
+      <c r="I34" t="n">
+        <v>2.46578123419643</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1139,6 +1451,15 @@
       <c r="F35" t="n">
         <v>52.2</v>
       </c>
+      <c r="G35" t="n">
+        <v>5.004152691454784</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0.9958473085452155</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0.9917118619367497</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1159,6 +1480,15 @@
       <c r="F36" t="n">
         <v>52</v>
       </c>
+      <c r="G36" t="n">
+        <v>5.151638601395248</v>
+      </c>
+      <c r="H36" t="n">
+        <v>-0.1516386013952484</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0.02299426543310704</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1179,6 +1509,15 @@
       <c r="F37" t="n">
         <v>34.2</v>
       </c>
+      <c r="G37" t="n">
+        <v>4.639775737484227</v>
+      </c>
+      <c r="H37" t="n">
+        <v>2.960224262515773</v>
+      </c>
+      <c r="I37" t="n">
+        <v>8.762927684387051</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1199,6 +1538,15 @@
       <c r="F38" t="n">
         <v>57.59999999999999</v>
       </c>
+      <c r="G38" t="n">
+        <v>5.082233467305619</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0.9177665326943814</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0.842295408533867</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1219,6 +1567,15 @@
       <c r="F39" t="n">
         <v>46.91999999999999</v>
       </c>
+      <c r="G39" t="n">
+        <v>5.134287317872841</v>
+      </c>
+      <c r="H39" t="n">
+        <v>-0.5342873178728418</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0.2854629380397551</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1239,6 +1596,15 @@
       <c r="F40" t="n">
         <v>49.68</v>
       </c>
+      <c r="G40" t="n">
+        <v>5.186341168440064</v>
+      </c>
+      <c r="H40" t="n">
+        <v>-0.5863411684400646</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0.3437959658076601</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1259,6 +1625,15 @@
       <c r="F41" t="n">
         <v>85.88</v>
       </c>
+      <c r="G41" t="n">
+        <v>5.229719377246083</v>
+      </c>
+      <c r="H41" t="n">
+        <v>2.370280622753917</v>
+      </c>
+      <c r="I41" t="n">
+        <v>5.618230230602697</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1279,6 +1654,15 @@
       <c r="F42" t="n">
         <v>77.7</v>
       </c>
+      <c r="G42" t="n">
+        <v>5.212368093723676</v>
+      </c>
+      <c r="H42" t="n">
+        <v>1.787631906276324</v>
+      </c>
+      <c r="I42" t="n">
+        <v>3.195627832337125</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1299,6 +1683,15 @@
       <c r="F43" t="n">
         <v>63.59999999999999</v>
       </c>
+      <c r="G43" t="n">
+        <v>5.168989884917656</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0.8310101150823437</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0.6905778113691701</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1319,6 +1712,15 @@
       <c r="F44" t="n">
         <v>59.40000000000001</v>
       </c>
+      <c r="G44" t="n">
+        <v>5.203692451962471</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0.1963075480375291</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0.03853665341650681</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1339,6 +1741,15 @@
       <c r="F45" t="n">
         <v>79.10000000000001</v>
       </c>
+      <c r="G45" t="n">
+        <v>5.229719377246083</v>
+      </c>
+      <c r="H45" t="n">
+        <v>1.770280622753917</v>
+      </c>
+      <c r="I45" t="n">
+        <v>3.133893483297998</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1359,6 +1770,15 @@
       <c r="F46" t="n">
         <v>56.56</v>
       </c>
+      <c r="G46" t="n">
+        <v>5.125611676111637</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0.4743883238883626</v>
+      </c>
+      <c r="I46" t="n">
+        <v>0.22504428184161</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1379,6 +1799,15 @@
       <c r="F47" t="n">
         <v>64</v>
       </c>
+      <c r="G47" t="n">
+        <v>5.116936034350434</v>
+      </c>
+      <c r="H47" t="n">
+        <v>1.283063965649567</v>
+      </c>
+      <c r="I47" t="n">
+        <v>1.646253139948393</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1399,6 +1828,15 @@
       <c r="F48" t="n">
         <v>77.59999999999999</v>
       </c>
+      <c r="G48" t="n">
+        <v>5.090909109066822</v>
+      </c>
+      <c r="H48" t="n">
+        <v>2.909090890933178</v>
+      </c>
+      <c r="I48" t="n">
+        <v>8.46280981171039</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1419,6 +1857,15 @@
       <c r="F49" t="n">
         <v>41.58</v>
       </c>
+      <c r="G49" t="n">
+        <v>4.795937289185894</v>
+      </c>
+      <c r="H49" t="n">
+        <v>1.804062710814105</v>
+      </c>
+      <c r="I49" t="n">
+        <v>3.254642264549938</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1439,6 +1886,15 @@
       <c r="F50" t="n">
         <v>62.40000000000001</v>
       </c>
+      <c r="G50" t="n">
+        <v>5.151638601395248</v>
+      </c>
+      <c r="H50" t="n">
+        <v>0.8483613986047516</v>
+      </c>
+      <c r="I50" t="n">
+        <v>0.7197170626426102</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1459,6 +1915,15 @@
       <c r="F51" t="n">
         <v>0</v>
       </c>
+      <c r="G51" t="n">
+        <v>4.249371858230057</v>
+      </c>
+      <c r="H51" t="n">
+        <v>2.750628141769943</v>
+      </c>
+      <c r="I51" t="n">
+        <v>7.565955174296771</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -1479,6 +1944,15 @@
       <c r="F52" t="n">
         <v>1.32</v>
       </c>
+      <c r="G52" t="n">
+        <v>4.30142570879728</v>
+      </c>
+      <c r="H52" t="n">
+        <v>-2.101425708797279</v>
+      </c>
+      <c r="I52" t="n">
+        <v>4.415990009594148</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -1499,6 +1973,15 @@
       <c r="F53" t="n">
         <v>24.4</v>
       </c>
+      <c r="G53" t="n">
+        <v>4.778586005663486</v>
+      </c>
+      <c r="H53" t="n">
+        <v>-0.7785860056634863</v>
+      </c>
+      <c r="I53" t="n">
+        <v>0.6061961682150224</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -1519,6 +2002,15 @@
       <c r="F54" t="n">
         <v>20.8</v>
       </c>
+      <c r="G54" t="n">
+        <v>4.943423199126358</v>
+      </c>
+      <c r="H54" t="n">
+        <v>-2.343423199126358</v>
+      </c>
+      <c r="I54" t="n">
+        <v>5.491632290203615</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -1539,6 +2031,15 @@
       <c r="F55" t="n">
         <v>16</v>
       </c>
+      <c r="G55" t="n">
+        <v>4.466262902260151</v>
+      </c>
+      <c r="H55" t="n">
+        <v>1.933737097739849</v>
+      </c>
+      <c r="I55" t="n">
+        <v>3.739339163175334</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -1559,6 +2060,15 @@
       <c r="F56" t="n">
         <v>25.2</v>
       </c>
+      <c r="G56" t="n">
+        <v>5.160314243156453</v>
+      </c>
+      <c r="H56" t="n">
+        <v>-2.760314243156453</v>
+      </c>
+      <c r="I56" t="n">
+        <v>7.619334720972382</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -1579,6 +2089,15 @@
       <c r="F57" t="n">
         <v>63.8</v>
       </c>
+      <c r="G57" t="n">
+        <v>5.203692451962471</v>
+      </c>
+      <c r="H57" t="n">
+        <v>0.5963075480375286</v>
+      </c>
+      <c r="I57" t="n">
+        <v>0.3555826918465295</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -1599,6 +2118,15 @@
       <c r="F58" t="n">
         <v>21.58</v>
       </c>
+      <c r="G58" t="n">
+        <v>4.96945012440997</v>
+      </c>
+      <c r="H58" t="n">
+        <v>-2.369450124409969</v>
+      </c>
+      <c r="I58" t="n">
+        <v>5.61429389206642</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -1619,6 +2147,15 @@
       <c r="F59" t="n">
         <v>44.64</v>
       </c>
+      <c r="G59" t="n">
+        <v>5.056206542022007</v>
+      </c>
+      <c r="H59" t="n">
+        <v>-0.2562065420220074</v>
+      </c>
+      <c r="I59" t="n">
+        <v>0.06564179217487466</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -1639,6 +2176,15 @@
       <c r="F60" t="n">
         <v>50.14</v>
       </c>
+      <c r="G60" t="n">
+        <v>5.195016810201268</v>
+      </c>
+      <c r="H60" t="n">
+        <v>-0.5950168102012681</v>
+      </c>
+      <c r="I60" t="n">
+        <v>0.3540450044220919</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -1659,6 +2205,15 @@
       <c r="F61" t="n">
         <v>60.32</v>
       </c>
+      <c r="G61" t="n">
+        <v>5.151638601395248</v>
+      </c>
+      <c r="H61" t="n">
+        <v>0.6483613986047514</v>
+      </c>
+      <c r="I61" t="n">
+        <v>0.4203725032007093</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -1679,6 +2234,15 @@
       <c r="F62" t="n">
         <v>72.59999999999999</v>
       </c>
+      <c r="G62" t="n">
+        <v>5.203692451962471</v>
+      </c>
+      <c r="H62" t="n">
+        <v>1.396307548037528</v>
+      </c>
+      <c r="I62" t="n">
+        <v>1.949674768706575</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -1699,6 +2263,15 @@
       <c r="F63" t="n">
         <v>39.9</v>
       </c>
+      <c r="G63" t="n">
+        <v>5.160314243156453</v>
+      </c>
+      <c r="H63" t="n">
+        <v>-1.360314243156453</v>
+      </c>
+      <c r="I63" t="n">
+        <v>1.850454840134313</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -1719,6 +2292,15 @@
       <c r="F64" t="n">
         <v>102.82</v>
       </c>
+      <c r="G64" t="n">
+        <v>5.090909109066822</v>
+      </c>
+      <c r="H64" t="n">
+        <v>5.509090890933177</v>
+      </c>
+      <c r="I64" t="n">
+        <v>30.35008244456291</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -1739,6 +2321,15 @@
       <c r="F65" t="n">
         <v>80.55999999999999</v>
       </c>
+      <c r="G65" t="n">
+        <v>5.168989884917656</v>
+      </c>
+      <c r="H65" t="n">
+        <v>2.431010115082343</v>
+      </c>
+      <c r="I65" t="n">
+        <v>5.909810179632668</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -1759,6 +2350,15 @@
       <c r="F66" t="n">
         <v>44.94</v>
       </c>
+      <c r="G66" t="n">
+        <v>5.17766552667886</v>
+      </c>
+      <c r="H66" t="n">
+        <v>-0.9776655266788596</v>
+      </c>
+      <c r="I66" t="n">
+        <v>0.955829882056252</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -1779,6 +2379,15 @@
       <c r="F67" t="n">
         <v>23.04</v>
       </c>
+      <c r="G67" t="n">
+        <v>4.804612930947098</v>
+      </c>
+      <c r="H67" t="n">
+        <v>-1.204612930947098</v>
+      </c>
+      <c r="I67" t="n">
+        <v>1.451092313404957</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -1799,6 +2408,15 @@
       <c r="F68" t="n">
         <v>15.04</v>
       </c>
+      <c r="G68" t="n">
+        <v>4.657127021006634</v>
+      </c>
+      <c r="H68" t="n">
+        <v>-1.457127021006634</v>
+      </c>
+      <c r="I68" t="n">
+        <v>2.123219155347666</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -1819,6 +2437,15 @@
       <c r="F69" t="n">
         <v>27.54</v>
       </c>
+      <c r="G69" t="n">
+        <v>4.691829588051449</v>
+      </c>
+      <c r="H69" t="n">
+        <v>0.7081704119485517</v>
+      </c>
+      <c r="I69" t="n">
+        <v>0.5015053323593814</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -1839,6 +2466,15 @@
       <c r="F70" t="n">
         <v>31.32</v>
       </c>
+      <c r="G70" t="n">
+        <v>4.752559080379875</v>
+      </c>
+      <c r="H70" t="n">
+        <v>0.6474409196201254</v>
+      </c>
+      <c r="I70" t="n">
+        <v>0.4191797443985537</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -1859,6 +2495,15 @@
       <c r="F71" t="n">
         <v>38.16</v>
       </c>
+      <c r="G71" t="n">
+        <v>5.168989884917656</v>
+      </c>
+      <c r="H71" t="n">
+        <v>-1.568989884917656</v>
+      </c>
+      <c r="I71" t="n">
+        <v>2.46172925897392</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -1879,6 +2524,15 @@
       <c r="F72" t="n">
         <v>28.48</v>
       </c>
+      <c r="G72" t="n">
+        <v>5.021503974977192</v>
+      </c>
+      <c r="H72" t="n">
+        <v>-1.821503974977192</v>
+      </c>
+      <c r="I72" t="n">
+        <v>3.317876730857712</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -1899,6 +2553,15 @@
       <c r="F73" t="n">
         <v>31.2</v>
       </c>
+      <c r="G73" t="n">
+        <v>4.92607191560395</v>
+      </c>
+      <c r="H73" t="n">
+        <v>-0.9260719156039503</v>
+      </c>
+      <c r="I73" t="n">
+        <v>0.8576091928703701</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -1919,6 +2582,15 @@
       <c r="F74" t="n">
         <v>11.88</v>
       </c>
+      <c r="G74" t="n">
+        <v>4.821964214469506</v>
+      </c>
+      <c r="H74" t="n">
+        <v>-3.021964214469506</v>
+      </c>
+      <c r="I74" t="n">
+        <v>9.132267713534297</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -1939,6 +2611,15 @@
       <c r="F75" t="n">
         <v>16.64</v>
       </c>
+      <c r="G75" t="n">
+        <v>4.700505229812653</v>
+      </c>
+      <c r="H75" t="n">
+        <v>-1.500505229812653</v>
+      </c>
+      <c r="I75" t="n">
+        <v>2.251515944695122</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -1959,6 +2640,15 @@
       <c r="F76" t="n">
         <v>4.76</v>
       </c>
+      <c r="G76" t="n">
+        <v>4.396857768170521</v>
+      </c>
+      <c r="H76" t="n">
+        <v>-1.596857768170521</v>
+      </c>
+      <c r="I76" t="n">
+        <v>2.549954731766537</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -1979,6 +2669,15 @@
       <c r="F77" t="n">
         <v>10.12</v>
       </c>
+      <c r="G77" t="n">
+        <v>4.44023597697654</v>
+      </c>
+      <c r="H77" t="n">
+        <v>0.1597640230234596</v>
+      </c>
+      <c r="I77" t="n">
+        <v>0.02552454305264053</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -1999,6 +2698,15 @@
       <c r="F78" t="n">
         <v>1.12</v>
       </c>
+      <c r="G78" t="n">
+        <v>4.318776992319687</v>
+      </c>
+      <c r="H78" t="n">
+        <v>-2.918776992319687</v>
+      </c>
+      <c r="I78" t="n">
+        <v>8.519259130894756</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -2019,6 +2727,15 @@
       <c r="F79" t="n">
         <v>0.96</v>
       </c>
+      <c r="G79" t="n">
+        <v>4.275398783513668</v>
+      </c>
+      <c r="H79" t="n">
+        <v>-1.075398783513668</v>
+      </c>
+      <c r="I79" t="n">
+        <v>1.156482543582677</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -2039,6 +2756,15 @@
       <c r="F80" t="n">
         <v>24</v>
       </c>
+      <c r="G80" t="n">
+        <v>4.683153946290245</v>
+      </c>
+      <c r="H80" t="n">
+        <v>0.1168460537097546</v>
+      </c>
+      <c r="I80" t="n">
+        <v>0.01365300026754287</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -2059,6 +2785,15 @@
       <c r="F81" t="n">
         <v>5.2</v>
       </c>
+      <c r="G81" t="n">
+        <v>4.362155201125706</v>
+      </c>
+      <c r="H81" t="n">
+        <v>-0.3621552011257059</v>
+      </c>
+      <c r="I81" t="n">
+        <v>0.1311563897024005</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -2079,6 +2814,15 @@
       <c r="F82" t="n">
         <v>34.5</v>
       </c>
+      <c r="G82" t="n">
+        <v>4.64845137924543</v>
+      </c>
+      <c r="H82" t="n">
+        <v>2.85154862075457</v>
+      </c>
+      <c r="I82" t="n">
+        <v>8.131329536527289</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -2099,6 +2843,15 @@
       <c r="F83" t="n">
         <v>7.2</v>
       </c>
+      <c r="G83" t="n">
+        <v>4.422884693454132</v>
+      </c>
+      <c r="H83" t="n">
+        <v>-0.8228846934541321</v>
+      </c>
+      <c r="I83" t="n">
+        <v>0.6771392187211009</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -2119,6 +2872,15 @@
       <c r="F84" t="n">
         <v>2.8</v>
       </c>
+      <c r="G84" t="n">
+        <v>4.310101350558483</v>
+      </c>
+      <c r="H84" t="n">
+        <v>-0.3101013505584831</v>
+      </c>
+      <c r="I84" t="n">
+        <v>0.09616284761819523</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -2139,6 +2901,15 @@
       <c r="F85" t="n">
         <v>4</v>
       </c>
+      <c r="G85" t="n">
+        <v>4.466262902260151</v>
+      </c>
+      <c r="H85" t="n">
+        <v>-2.866262902260151</v>
+      </c>
+      <c r="I85" t="n">
+        <v>8.215463024872786</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -2159,6 +2930,15 @@
       <c r="F86" t="n">
         <v>26.52</v>
       </c>
+      <c r="G86" t="n">
+        <v>5.134287317872841</v>
+      </c>
+      <c r="H86" t="n">
+        <v>-2.534287317872841</v>
+      </c>
+      <c r="I86" t="n">
+        <v>6.42261220953112</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -2179,6 +2959,15 @@
       <c r="F87" t="n">
         <v>39.52</v>
       </c>
+      <c r="G87" t="n">
+        <v>4.908720632081543</v>
+      </c>
+      <c r="H87" t="n">
+        <v>0.2912793679184569</v>
+      </c>
+      <c r="I87" t="n">
+        <v>0.08484367017497577</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -2199,6 +2988,15 @@
       <c r="F88" t="n">
         <v>64.59999999999999</v>
       </c>
+      <c r="G88" t="n">
+        <v>4.986801407932377</v>
+      </c>
+      <c r="H88" t="n">
+        <v>2.613198592067622</v>
+      </c>
+      <c r="I88" t="n">
+        <v>6.828806881584203</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -2219,6 +3017,15 @@
       <c r="F89" t="n">
         <v>39.9</v>
       </c>
+      <c r="G89" t="n">
+        <v>5.160314243156453</v>
+      </c>
+      <c r="H89" t="n">
+        <v>-1.360314243156453</v>
+      </c>
+      <c r="I89" t="n">
+        <v>1.850454840134313</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -2239,6 +3046,15 @@
       <c r="F90" t="n">
         <v>35.28</v>
       </c>
+      <c r="G90" t="n">
+        <v>5.099584750828027</v>
+      </c>
+      <c r="H90" t="n">
+        <v>-1.499584750828026</v>
+      </c>
+      <c r="I90" t="n">
+        <v>2.248754424915954</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -2259,6 +3075,15 @@
       <c r="F91" t="n">
         <v>10.8</v>
       </c>
+      <c r="G91" t="n">
+        <v>4.483614185782558</v>
+      </c>
+      <c r="H91" t="n">
+        <v>-0.4836141857825584</v>
+      </c>
+      <c r="I91" t="n">
+        <v>0.2338826806901269</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -2279,6 +3104,15 @@
       <c r="F92" t="n">
         <v>21.84</v>
       </c>
+      <c r="G92" t="n">
+        <v>5.038855258499599</v>
+      </c>
+      <c r="H92" t="n">
+        <v>-2.638855258499599</v>
+      </c>
+      <c r="I92" t="n">
+        <v>6.963557075310987</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -2299,6 +3133,15 @@
       <c r="F93" t="n">
         <v>35.7</v>
       </c>
+      <c r="G93" t="n">
+        <v>5.160314243156453</v>
+      </c>
+      <c r="H93" t="n">
+        <v>-1.760314243156453</v>
+      </c>
+      <c r="I93" t="n">
+        <v>3.098706234659476</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -2319,6 +3162,15 @@
       <c r="F94" t="n">
         <v>37.08000000000001</v>
       </c>
+      <c r="G94" t="n">
+        <v>5.142962959634045</v>
+      </c>
+      <c r="H94" t="n">
+        <v>-1.542962959634045</v>
+      </c>
+      <c r="I94" t="n">
+        <v>2.380734694802651</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -2339,6 +3191,15 @@
       <c r="F95" t="n">
         <v>20</v>
       </c>
+      <c r="G95" t="n">
+        <v>5.116936034350434</v>
+      </c>
+      <c r="H95" t="n">
+        <v>-3.116936034350434</v>
+      </c>
+      <c r="I95" t="n">
+        <v>9.715290242232207</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -2359,6 +3220,15 @@
       <c r="F96" t="n">
         <v>10.54</v>
       </c>
+      <c r="G96" t="n">
+        <v>4.518316752827373</v>
+      </c>
+      <c r="H96" t="n">
+        <v>-1.118316752827373</v>
+      </c>
+      <c r="I96" t="n">
+        <v>1.250632359654361</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -2379,6 +3249,15 @@
       <c r="F97" t="n">
         <v>33.84</v>
       </c>
+      <c r="G97" t="n">
+        <v>5.064882183783211</v>
+      </c>
+      <c r="H97" t="n">
+        <v>-1.464882183783211</v>
+      </c>
+      <c r="I97" t="n">
+        <v>2.145879812365468</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -2399,6 +3278,15 @@
       <c r="F98" t="n">
         <v>32.64</v>
       </c>
+      <c r="G98" t="n">
+        <v>5.134287317872841</v>
+      </c>
+      <c r="H98" t="n">
+        <v>-1.934287317872841</v>
+      </c>
+      <c r="I98" t="n">
+        <v>3.74146742808371</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -2419,6 +3307,15 @@
       <c r="F99" t="n">
         <v>32.32</v>
       </c>
+      <c r="G99" t="n">
+        <v>5.125611676111637</v>
+      </c>
+      <c r="H99" t="n">
+        <v>-1.925611676111637</v>
+      </c>
+      <c r="I99" t="n">
+        <v>3.707980327177467</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -2439,6 +3336,15 @@
       <c r="F100" t="n">
         <v>28.8</v>
       </c>
+      <c r="G100" t="n">
+        <v>5.082233467305619</v>
+      </c>
+      <c r="H100" t="n">
+        <v>-2.082233467305619</v>
+      </c>
+      <c r="I100" t="n">
+        <v>4.335696212367579</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -2458,6 +3364,15 @@
       </c>
       <c r="F101" t="n">
         <v>2.52</v>
+      </c>
+      <c r="G101" t="n">
+        <v>4.431560335215336</v>
+      </c>
+      <c r="H101" t="n">
+        <v>-3.231560335215335</v>
+      </c>
+      <c r="I101" t="n">
+        <v>10.44298220013705</v>
       </c>
     </row>
   </sheetData>

</xml_diff>